<commit_message>
Script updated for registration module
</commit_message>
<xml_diff>
--- a/src/main/resources/UserRegistration_Field_Values.xlsx
+++ b/src/main/resources/UserRegistration_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Cleanup_Projects\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Santosh\REIProject\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F57F245C-9349-4AD8-8A44-292BF2A1671D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6ED59F4-4C70-4248-88BA-F4535E6C7162}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="21" activeTab="23" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="21" activeTab="22" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CreationWithAllDetails" sheetId="1" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="107">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -173,12 +173,6 @@
     <t>Mr.</t>
   </si>
   <si>
-    <t>fieldPrimaryRepFirstName__c</t>
-  </si>
-  <si>
-    <t>fieldPrimaryRepLastName__c</t>
-  </si>
-  <si>
     <t>User</t>
   </si>
   <si>
@@ -266,25 +260,7 @@
     <t>DC</t>
   </si>
   <si>
-    <t>fieldPrimaryRepAddress1__c</t>
-  </si>
-  <si>
     <t>Automation</t>
-  </si>
-  <si>
-    <t>fieldPrimaryRepCity__c</t>
-  </si>
-  <si>
-    <t>fieldPrimaryRepState__c</t>
-  </si>
-  <si>
-    <t>fieldPrimaryRepZipCode__c</t>
-  </si>
-  <si>
-    <t>fieldPrimaryRepCountry__c</t>
-  </si>
-  <si>
-    <t>fieldPrimaryRepPhone__c</t>
   </si>
   <si>
     <t>Automation Representative</t>
@@ -867,10 +843,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="32.44140625" customWidth="1"/>
-    <col min="3" max="3" width="51.21875" customWidth="1"/>
+    <col min="2" max="2" width="32.453125" customWidth="1"/>
+    <col min="3" max="3" width="51.1796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -892,7 +868,7 @@
         <v>8</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -900,10 +876,10 @@
         <v>3</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="C3" s="19" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -911,7 +887,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="C4" s="19" t="s">
         <v>24</v>
@@ -922,10 +898,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="C5" s="20" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -933,7 +909,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="C6" s="19" t="s">
         <v>23</v>
@@ -944,10 +920,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -955,7 +931,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C8" s="19" t="s">
         <v>22</v>
@@ -966,10 +942,10 @@
         <v>3</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -977,10 +953,10 @@
         <v>3</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -988,7 +964,7 @@
         <v>3</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="C11" s="19">
         <v>20171</v>
@@ -999,7 +975,7 @@
         <v>3</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="C12" s="19" t="s">
         <v>24</v>
@@ -1017,7 +993,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="7" t="s">
@@ -1079,7 +1055,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C6" t="s">
         <v>6</v>
@@ -1090,10 +1066,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C7" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1104,7 +1080,7 @@
         <v>35</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -1115,7 +1091,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="7" t="s">
@@ -1177,7 +1153,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C6" t="s">
         <v>6</v>
@@ -1188,10 +1164,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -1202,9 +1178,9 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="28.44140625" customWidth="1"/>
+    <col min="2" max="2" width="28.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1267,7 +1243,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C6" t="s">
         <v>5</v>
@@ -1278,7 +1254,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C7" t="s">
         <v>6</v>
@@ -1289,7 +1265,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -1303,10 +1279,10 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="20.44140625" customWidth="1"/>
-    <col min="3" max="3" width="17.77734375" customWidth="1"/>
+    <col min="2" max="2" width="20.453125" customWidth="1"/>
+    <col min="3" max="3" width="17.81640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1339,9 +1315,9 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="23.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1375,9 +1351,9 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="18.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1410,9 +1386,9 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="20.44140625" customWidth="1"/>
+    <col min="2" max="2" width="20.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1445,10 +1421,10 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="13.5546875" customWidth="1"/>
-    <col min="3" max="3" width="19.21875" customWidth="1"/>
+    <col min="2" max="2" width="13.54296875" customWidth="1"/>
+    <col min="3" max="3" width="19.1796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1492,10 +1468,10 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="29.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.77734375" customWidth="1"/>
+    <col min="2" max="2" width="29.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.81640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1572,7 +1548,7 @@
         <v>21</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -1587,10 +1563,10 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="25.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="36.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1612,7 +1588,7 @@
         <v>26</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1646,9 +1622,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B828E63F-C4C2-4AE0-A0E9-A1CABDF6D980}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="27.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.54296875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="37" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1668,10 +1644,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="24" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="C2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1679,7 +1655,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="24" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -1693,10 +1669,10 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="28.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="36.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1718,7 +1694,7 @@
         <v>26</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1774,10 +1750,10 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1200-000000000000}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="22.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1844,10 +1820,10 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1300-000000000000}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="22.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1925,9 +1901,9 @@
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1400-000000000000}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="39.5546875" customWidth="1"/>
+    <col min="2" max="2" width="39.54296875" customWidth="1"/>
     <col min="3" max="3" width="45" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1947,10 +1923,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>41</v>
+        <v>95</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1958,10 +1934,10 @@
         <v>3</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>42</v>
+        <v>96</v>
       </c>
       <c r="C3" s="19" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1969,10 +1945,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>72</v>
+        <v>97</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1980,10 +1956,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>74</v>
+        <v>98</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1991,10 +1967,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>75</v>
+        <v>99</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -2002,7 +1978,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>76</v>
+        <v>100</v>
       </c>
       <c r="C7" s="19">
         <v>20301</v>
@@ -2013,10 +1989,10 @@
         <v>3</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -2024,7 +2000,7 @@
         <v>3</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>78</v>
+        <v>102</v>
       </c>
       <c r="C9" s="19" t="s">
         <v>24</v>
@@ -2039,9 +2015,9 @@
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A47B17BA-F990-45EB-8B28-07CF77412B89}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="3" width="25.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="25.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2060,10 +2036,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -2071,10 +2047,10 @@
         <v>3</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -2082,10 +2058,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -2093,10 +2069,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -2104,10 +2080,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -2115,7 +2091,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="C7" s="8">
         <v>20301</v>
@@ -2126,10 +2102,10 @@
         <v>3</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -2137,7 +2113,7 @@
         <v>3</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="C9" s="8">
         <v>7890368902</v>
@@ -2151,11 +2127,11 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2174,7 +2150,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="C2" s="19" t="s">
         <v>40</v>
@@ -2185,10 +2161,10 @@
         <v>3</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="C3" s="19" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -2196,10 +2172,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -2207,10 +2183,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -2218,10 +2194,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -2229,10 +2205,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -2240,7 +2216,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="C8" s="19">
         <v>20301</v>
@@ -2251,10 +2227,10 @@
         <v>3</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -2262,7 +2238,7 @@
         <v>3</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="C10" s="19" t="s">
         <v>24</v>
@@ -2273,10 +2249,10 @@
         <v>3</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -2291,11 +2267,11 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2317,7 +2293,7 @@
         <v>8</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -2325,10 +2301,10 @@
         <v>3</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C3" s="19" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -2347,10 +2323,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C5" s="20" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -2358,10 +2334,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -2380,10 +2356,10 @@
         <v>3</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -2402,10 +2378,10 @@
         <v>3</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -2413,10 +2389,10 @@
         <v>3</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -2435,7 +2411,7 @@
         <v>3</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C13" s="19" t="s">
         <v>24</v>
@@ -2452,10 +2428,10 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2476,7 +2452,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="C2" s="17" t="s">
         <v>6</v>
@@ -2489,10 +2465,10 @@
         <v>3</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="C3" s="19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D3" s="16"/>
       <c r="E3" s="16"/>
@@ -2502,10 +2478,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D4" s="16"/>
       <c r="E4" s="16"/>
@@ -2515,10 +2491,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
@@ -2528,7 +2504,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="C6" s="19">
         <v>20301</v>
@@ -2541,7 +2517,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="C7" s="19">
         <v>1234</v>
@@ -2554,7 +2530,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="C8" s="19" t="s">
         <v>24</v>
@@ -2571,7 +2547,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6449BFBB-D262-4256-B30F-8A2BD0B132FE}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2580,9 +2556,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="29.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.54296875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="34" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2660,7 +2636,7 @@
         <v>21</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -2675,11 +2651,11 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="14.21875" customWidth="1"/>
-    <col min="2" max="2" width="20.77734375" customWidth="1"/>
-    <col min="3" max="3" width="43.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.1796875" customWidth="1"/>
+    <col min="2" max="2" width="20.81640625" customWidth="1"/>
+    <col min="3" max="3" width="43.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2701,7 +2677,7 @@
         <v>8</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -2745,7 +2721,7 @@
         <v>12</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -2770,7 +2746,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
@@ -2810,10 +2786,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Script updated for registration modules
</commit_message>
<xml_diff>
--- a/src/main/resources/UserRegistration_Field_Values.xlsx
+++ b/src/main/resources/UserRegistration_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Santosh\REIProject\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6ED59F4-4C70-4248-88BA-F4535E6C7162}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0700FC91-25E7-4C10-8DF3-C395017E583D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="21" activeTab="22" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="22" activeTab="22" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CreationWithAllDetails" sheetId="1" r:id="rId1"/>
@@ -278,9 +278,6 @@
     <t>SameAsOrganizationAddress__c</t>
   </si>
   <si>
-    <t>PaymentAddressLine1__c</t>
-  </si>
-  <si>
     <t>PaymentAddressCity__c</t>
   </si>
   <si>
@@ -369,6 +366,9 @@
   </si>
   <si>
     <t>EffectiveDate__c</t>
+  </si>
+  <si>
+    <t>PaymentAddressline1__c</t>
   </si>
 </sst>
 </file>
@@ -876,10 +876,10 @@
         <v>3</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C3" s="19" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -887,7 +887,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C4" s="19" t="s">
         <v>24</v>
@@ -898,7 +898,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C5" s="20" t="s">
         <v>57</v>
@@ -909,7 +909,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C6" s="19" t="s">
         <v>23</v>
@@ -920,10 +920,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -931,7 +931,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C8" s="19" t="s">
         <v>22</v>
@@ -942,10 +942,10 @@
         <v>3</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -953,7 +953,7 @@
         <v>3</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C10" s="19" t="s">
         <v>65</v>
@@ -964,7 +964,7 @@
         <v>3</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C11" s="19">
         <v>20171</v>
@@ -975,7 +975,7 @@
         <v>3</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C12" s="19" t="s">
         <v>24</v>
@@ -1644,7 +1644,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="24" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C2" t="s">
         <v>59</v>
@@ -1655,7 +1655,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="24" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -1923,7 +1923,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C2" s="19" t="s">
         <v>74</v>
@@ -1934,7 +1934,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C3" s="19" t="s">
         <v>41</v>
@@ -1945,7 +1945,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C4" s="19" t="s">
         <v>71</v>
@@ -1956,7 +1956,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C5" s="19" t="s">
         <v>68</v>
@@ -1967,7 +1967,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C6" s="19" t="s">
         <v>69</v>
@@ -1978,7 +1978,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C7" s="19">
         <v>20301</v>
@@ -1989,7 +1989,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C8" s="19" t="s">
         <v>65</v>
@@ -2000,7 +2000,7 @@
         <v>3</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C9" s="19" t="s">
         <v>24</v>
@@ -2036,7 +2036,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C2" s="8" t="s">
         <v>74</v>
@@ -2047,7 +2047,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>41</v>
@@ -2058,7 +2058,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>71</v>
@@ -2069,7 +2069,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>68</v>
@@ -2080,10 +2080,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -2091,7 +2091,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C7" s="8">
         <v>20301</v>
@@ -2102,7 +2102,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>65</v>
@@ -2113,7 +2113,7 @@
         <v>3</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C9" s="8">
         <v>7890368902</v>
@@ -2150,7 +2150,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C2" s="19" t="s">
         <v>40</v>
@@ -2161,7 +2161,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C3" s="19" t="s">
         <v>70</v>
@@ -2172,7 +2172,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C4" s="19" t="s">
         <v>41</v>
@@ -2183,7 +2183,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C5" s="19" t="s">
         <v>71</v>
@@ -2194,7 +2194,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C6" s="19" t="s">
         <v>68</v>
@@ -2205,7 +2205,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C7" s="19" t="s">
         <v>69</v>
@@ -2216,7 +2216,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C8" s="19">
         <v>20301</v>
@@ -2227,7 +2227,7 @@
         <v>3</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C9" s="19" t="s">
         <v>65</v>
@@ -2238,7 +2238,7 @@
         <v>3</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C10" s="19" t="s">
         <v>24</v>
@@ -2249,7 +2249,7 @@
         <v>3</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>72</v>
@@ -2304,7 +2304,7 @@
         <v>55</v>
       </c>
       <c r="C3" s="19" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -2465,7 +2465,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>76</v>
+        <v>106</v>
       </c>
       <c r="C3" s="19" t="s">
         <v>67</v>
@@ -2478,7 +2478,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C4" s="19" t="s">
         <v>68</v>
@@ -2491,10 +2491,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
@@ -2504,7 +2504,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C6" s="19">
         <v>20301</v>
@@ -2517,7 +2517,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C7" s="19">
         <v>1234</v>
@@ -2530,7 +2530,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C8" s="19" t="s">
         <v>24</v>

</xml_diff>